<commit_message>
Map Buzzoola party addresses and lock partner dumps with header checks.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Шаблон/Шаблон загрузки данных от DSP (2).xlsx
+++ b/Шаблон/Шаблон загрузки данных от DSP (2).xlsx
@@ -46,8 +46,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -417,107 +420,107 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>ERID</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Номер изначального договора</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Дата изначального договора</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Тип договора</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Предмет договора</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Вид деятельности</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Тип заказчика</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Заказчик</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Адрес заказчика</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>ИНН заказчика или его аналог</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Рег.номер заказчика</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>ОКСМ заказчика</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Тип исполнителя</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Исполнитель</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Адрес исполнителя</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>ИНН исполнителя или его аналог</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Рег.номер исполнителя</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>ОКСМ исполнителя</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Включая НДС</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="2" t="inlineStr">
         <is>
           <t>Показы</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="3" t="inlineStr">
         <is>
           <t>Сумма</t>
         </is>

</xml_diff>